<commit_message>
Skipped weeks kept valid, no privacy consent, Excel export
- Subscriptions: a lost week can be kept valid with one tap ("Non farla
  perdere", with Annulla). It stays "da recuperare" and counts as a
  lesson left until a later week has a second lesson; the "+" and the
  classes record that lesson without asking for confirmation.
- No privacy consent in the app (form, client page, import, demo data):
  the app holds no health data; the postural assessment (old M7) stays
  outside the app.
- Altro → "Esporta i dati": one Excel file with clients, packages,
  lessons, appointments, classes and prices; the Clienti sheet can be
  imported again. Automatic backup planned in M5.
- Spec: Excel may be cleaned by Claude in chat (never in the repo).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q45KoBviJaHGSidLZnkXBh
</commit_message>
<xml_diff>
--- a/public/esempio-clienti.xlsx
+++ b/public/esempio-clienti.xlsx
@@ -37,9 +37,6 @@
     <t>Note</t>
   </si>
   <si>
-    <t>Consenso privacy</t>
-  </si>
-  <si>
     <t>Laura</t>
   </si>
   <si>
@@ -55,10 +52,7 @@
     <t>Fisio</t>
   </si>
   <si>
-    <t>Dolore cervicale</t>
-  </si>
-  <si>
-    <t>Sì</t>
+    <t>Preferisce la sera</t>
   </si>
   <si>
     <t>Giorgio</t>
@@ -127,9 +121,6 @@
     <t>posturale</t>
   </si>
   <si>
-    <t>sì</t>
-  </si>
-  <si>
     <t>Elisa</t>
   </si>
   <si>
@@ -145,10 +136,7 @@
     <t>yoga</t>
   </si>
   <si>
-    <t>Consenso da far firmare</t>
-  </si>
-  <si>
-    <t>No</t>
+    <t>Chiede sempre il martedì</t>
   </si>
   <si>
     <t>Giulia</t>
@@ -221,7 +209,6 @@
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="24" customWidth="1"/>
     <col min="7" max="7" width="34" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -246,125 +233,107 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
       </c>
       <c r="E2" s="2">
         <v>32216</v>
       </c>
       <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
         <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
         <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>17</v>
       </c>
       <c r="E3" s="2">
         <v>27700</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
         <v>19</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>20</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>22</v>
-      </c>
-      <c r="E4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
         <v>25</v>
       </c>
-      <c r="B5" t="s">
+      <c r="F5" t="s">
         <v>26</v>
       </c>
-      <c r="D5" t="s">
+      <c r="G5" t="s">
         <v>27</v>
-      </c>
-      <c r="F5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H5" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
         <v>30</v>
-      </c>
-      <c r="B6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" t="s">
-        <v>32</v>
       </c>
       <c r="E6" s="2">
         <v>33806</v>
       </c>
       <c r="F6" t="s">
-        <v>33</v>
-      </c>
-      <c r="H6" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C7">
         <v>3000000206</v>
@@ -373,64 +342,52 @@
         <v>25233</v>
       </c>
       <c r="F7" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" t="s">
         <v>38</v>
       </c>
-      <c r="B8" t="s">
+      <c r="F8" t="s">
         <v>39</v>
       </c>
-      <c r="C8" t="s">
+      <c r="G8" t="s">
         <v>40</v>
-      </c>
-      <c r="D8" t="s">
-        <v>41</v>
-      </c>
-      <c r="F8" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H8" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="F9" t="s">
-        <v>12</v>
-      </c>
-      <c r="H9" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F10" t="s">
-        <v>24</v>
-      </c>
-      <c r="H10" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>